<commit_message>
Fix issue that there is space in curve name.
</commit_message>
<xml_diff>
--- a/ConfigTable/DT_BattleParam_DefaultCharacter.xlsx
+++ b/ConfigTable/DT_BattleParam_DefaultCharacter.xlsx
@@ -33,9 +33,6 @@
     <t>Dexterity</t>
   </si>
   <si>
-    <t xml:space="preserve">Agility </t>
-  </si>
-  <si>
     <t>HP</t>
   </si>
   <si>
@@ -43,6 +40,9 @@
   </si>
   <si>
     <t>Character Parameter</t>
+  </si>
+  <si>
+    <t>Agility</t>
   </si>
 </sst>
 </file>
@@ -412,7 +412,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="33.75">
       <c r="A1" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -429,19 +429,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>